<commit_message>
Upload 2 files via dashboard admin
- October_26_Utilities_Tracking.xlsx
- CBG OEE (Availability and Utilization) Calculation- 2026.xlsx
</commit_message>
<xml_diff>
--- a/data/raw/CBG OEE (Availability and Utilization) Calculation- 2026.xlsx
+++ b/data/raw/CBG OEE (Availability and Utilization) Calculation- 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ansamcal.sharepoint.com/sites/CBGPackagingLineOperations/Shared Documents/General/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7ED3841B-C042-4E2E-BA0F-D396709C4721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B88A24E-AC18-4C82-B38B-4FA618077E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4254,7 +4254,7 @@
                     <c:extLst>
                       <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                       <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                        <c16:uniqueId val="{00000012-112F-4FBE-BB51-673234708240}"/>
+                        <c16:uniqueId val="{00000012-246F-4461-8926-B489BF549057}"/>
                       </c:ext>
                     </c:extLst>
                   </c15:dLbl>

</xml_diff>

<commit_message>
Upload CBG OEE (Availability and Utilization) Calculation- 2026.xlsx via dashboard admin
</commit_message>
<xml_diff>
--- a/data/raw/CBG OEE (Availability and Utilization) Calculation- 2026.xlsx
+++ b/data/raw/CBG OEE (Availability and Utilization) Calculation- 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ansamcal.sharepoint.com/sites/CBGPackagingLineOperations/Shared Documents/General/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB611B8A-73EB-462C-8D52-A167D6A0FFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C2D49DA-456B-4476-B16A-18ACEBF69628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" firstSheet="10" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January 2026 (w Utilization)" sheetId="39" r:id="rId1"/>
@@ -984,7 +984,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="161">
   <si>
     <t>OEE Calculation</t>
   </si>
@@ -1466,6 +1466,9 @@
   </si>
   <si>
     <t>Starmalt to Vitamalt Classic</t>
+  </si>
+  <si>
+    <t>Carib Amber tp Stag</t>
   </si>
   <si>
     <t>January</t>
@@ -2928,13 +2931,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.7947444035555471</c:v>
+                  <c:v>0.79822557953444684</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.86786296900537074</c:v>
+                  <c:v>0.86731919521526935</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.91778966131907314</c:v>
+                  <c:v>0.92238774297597825</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.99777624354757888</c:v>
@@ -3084,13 +3087,13 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.2052555964444529</c:v>
+                  <c:v>0.20177442046555316</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.13213703099462926</c:v>
+                  <c:v>0.13268080478473065</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.2210338680926864E-2</c:v>
+                  <c:v>7.7612257024021747E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2.2237564524211217E-3</c:v>
@@ -4254,7 +4257,7 @@
                     <c:extLst>
                       <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                       <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                        <c16:uniqueId val="{00000012-9018-4ADB-B2E7-A8C693DDDE96}"/>
+                        <c16:uniqueId val="{00000012-0200-427D-93E2-DEFFF7C4DADB}"/>
                       </c:ext>
                     </c:extLst>
                   </c15:dLbl>
@@ -22985,18 +22988,24 @@
       </c>
     </row>
     <row r="8" spans="1:24">
-      <c r="A8" s="29"/>
+      <c r="A8" s="29" t="s">
+        <v>145</v>
+      </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8" t="str">
+      <c r="E8" s="7">
+        <v>10</v>
+      </c>
+      <c r="F8" s="7">
+        <v>12</v>
+      </c>
+      <c r="G8" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="47"/>
@@ -23010,14 +23019,23 @@
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N8" s="7"/>
-      <c r="O8" s="15"/>
+      <c r="N8" s="7">
+        <v>17000</v>
+      </c>
+      <c r="O8" s="15">
+        <f>AVERAGE(15000,15000,16000,15000,14000,16000,18000,18000,18000,18000,15500,15500,15500,15500)</f>
+        <v>16071.428571428571</v>
+      </c>
       <c r="P8" s="9" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
+      <c r="Q8" s="15">
+        <v>5473</v>
+      </c>
+      <c r="R8" s="15">
+        <v>24</v>
+      </c>
       <c r="S8" s="7"/>
       <c r="T8" s="5"/>
       <c r="U8" s="10" t="str">
@@ -24586,15 +24604,15 @@
       </c>
       <c r="E38" s="33">
         <f>SUM(E3:E37)</f>
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F38" s="33">
         <f>SUM(F3:F37)</f>
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="G38" s="33">
         <f>SUM(G3:G37)</f>
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="H38" s="33">
         <f>SUM(H2:H37)</f>
@@ -24606,7 +24624,7 @@
       </c>
       <c r="J38" s="34">
         <f>(D38-G38-H38-I38)/D38</f>
-        <v>0.86786296900537074</v>
+        <v>0.86731919521526935</v>
       </c>
       <c r="K38" s="35">
         <f>SUM(K3:K37)</f>
@@ -24618,7 +24636,7 @@
       </c>
       <c r="M38" s="36">
         <f>(D38-G38-H38-I38-E38-K38-L38)/D38</f>
-        <v>0.80152256661300547</v>
+        <v>0.7982599238723973</v>
       </c>
       <c r="N38" s="37">
         <f>AVERAGE(N3:N37)</f>
@@ -24626,15 +24644,15 @@
       </c>
       <c r="O38" s="38">
         <f>AVERAGE(O3:O37)</f>
-        <v>15602.424242424244</v>
+        <v>15680.591630591631</v>
       </c>
       <c r="P38" s="34">
         <f>O38/N38</f>
-        <v>0.91778966131907314</v>
+        <v>0.92238774297597825</v>
       </c>
       <c r="Q38" s="37">
         <f>SUM(Q3:Q35)</f>
-        <v>26297</v>
+        <v>31770</v>
       </c>
       <c r="R38" s="37"/>
       <c r="S38" s="32"/>
@@ -24646,11 +24664,11 @@
       </c>
       <c r="W38" s="41">
         <f>V38*P38*J38</f>
-        <v>0.7947444035555471</v>
+        <v>0.79822557953444684</v>
       </c>
       <c r="X38" s="42">
         <f>V38*P38*M38</f>
-        <v>0.7339932649381451</v>
+        <v>0.73466780611723492</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="28.5">
@@ -24673,7 +24691,7 @@
       <c r="S41" s="67"/>
       <c r="T41" s="46">
         <f>AVERAGE('January 2026 (w Utilization)'!X38,'February 2026 (w Utilization) '!X38,'March 2026 (w Utilization'!X38,'April 2026 (w Utilization) '!X38,'May 2026 (w Utilization)'!X38,'June 2026 (w Utilization)'!X38,'June 2026 (w Utilization)'!X38,'July 2026 (w Utilization)'!X38,'August 2026 (w Utilization)'!X38,'September 2026 (w Utilization)'!X38,'October 2026 (w Utilization) '!X38)</f>
-        <v>0.58332931505680186</v>
+        <v>0.58339063698217364</v>
       </c>
       <c r="U41" s="22"/>
     </row>
@@ -24713,11 +24731,11 @@
       </c>
       <c r="D47" s="16">
         <f>W38</f>
-        <v>0.7947444035555471</v>
+        <v>0.79822557953444684</v>
       </c>
       <c r="E47" s="18">
         <f>100%-D47</f>
-        <v>0.2052555964444529</v>
+        <v>0.20177442046555316</v>
       </c>
     </row>
     <row r="48" spans="1:24">
@@ -24726,11 +24744,11 @@
       </c>
       <c r="D48" s="16">
         <f>J38</f>
-        <v>0.86786296900537074</v>
+        <v>0.86731919521526935</v>
       </c>
       <c r="E48" s="18">
         <f>100%-D48</f>
-        <v>0.13213703099462926</v>
+        <v>0.13268080478473065</v>
       </c>
     </row>
     <row r="49" spans="3:5">
@@ -24739,11 +24757,11 @@
       </c>
       <c r="D49" s="16">
         <f>P38</f>
-        <v>0.91778966131907314</v>
+        <v>0.92238774297597825</v>
       </c>
       <c r="E49" s="18">
         <f>100%-D49</f>
-        <v>8.2210338680926864E-2</v>
+        <v>7.7612257024021747E-2</v>
       </c>
     </row>
     <row r="50" spans="3:5">
@@ -24793,51 +24811,51 @@
         <v>24</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H3" s="24" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I3" s="24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J3" s="24" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="L3" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M3" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N3" s="24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O3" s="23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P3" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="2:18">
       <c r="B4" s="23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C4" s="26">
         <f>'January 2026 (w Utilization)'!W38</f>
@@ -24877,7 +24895,7 @@
       </c>
       <c r="L4" s="26">
         <f>'October 2026 (w Utilization) '!W38</f>
-        <v>0.7947444035555471</v>
+        <v>0.79822557953444684</v>
       </c>
       <c r="M4" s="26" t="e">
         <f>'November 2025 (w Utilization)'!W38</f>
@@ -24897,7 +24915,7 @@
     </row>
     <row r="5" spans="2:18">
       <c r="B5" s="23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C5" s="25">
         <f>C4</f>
@@ -24937,7 +24955,7 @@
       </c>
       <c r="L5" s="25">
         <f>AVERAGE($C$4:L4)</f>
-        <v>0.6876669913132446</v>
+        <v>0.6880151089111346</v>
       </c>
       <c r="M5" s="25" t="e">
         <f>AVERAGE($C$4:M4)</f>
@@ -24965,46 +24983,46 @@
     </row>
     <row r="32" spans="3:16" ht="18.75">
       <c r="C32" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E32" s="24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F32" s="24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G32" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H32" s="24" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J32" s="24" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K32" s="24" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="L32" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M32" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N32" s="24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O32" s="23" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P32" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="2:17" ht="30">
@@ -51957,18 +51975,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -52116,11 +52134,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A0221E9-7351-4007-92F0-8B6A656CD9C4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77075DFF-DEDE-4E50-8ADC-F3E74E8E52C5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77075DFF-DEDE-4E50-8ADC-F3E74E8E52C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A0221E9-7351-4007-92F0-8B6A656CD9C4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>